<commit_message>
Mettre a jour les donnees materiaux (xlsx + .dat regeneres)
Material_intensities.xlsx, Material_limits.xlsx et Material_intensity/limits/recycling.dat.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/critical_materials/excel_files/Material_intensities.xlsx
+++ b/projects/critical_materials/excel_files/Material_intensities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Paolo/Documents/PdM_code/EnergyScope-Quebec/projects/critical_materials/excel_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82F4D53-204B-A849-B17D-FF5B199CA5F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7581429C-EFEB-FB41-9E0B-BD870AB49239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="36020" windowHeight="20960" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table of content" sheetId="1" r:id="rId1"/>
@@ -4853,6 +4853,13 @@
     <xf numFmtId="0" fontId="16" fillId="38" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="39" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -4875,18 +4882,11 @@
     <xf numFmtId="0" fontId="0" fillId="39" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="39" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -23539,7 +23539,7 @@
       </c>
       <c r="G388" s="4"/>
     </row>
-    <row r="389" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="389" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A389" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23562,7 +23562,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="390" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="390" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A390" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23585,7 +23585,7 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="391" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="391" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A391" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23606,7 +23606,7 @@
       </c>
       <c r="G391" s="4"/>
     </row>
-    <row r="392" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="392" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A392" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23627,7 +23627,7 @@
       </c>
       <c r="G392" s="4"/>
     </row>
-    <row r="393" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="393" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A393" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23650,7 +23650,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="394" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="394" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A394" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23671,7 +23671,7 @@
       </c>
       <c r="G394" s="4"/>
     </row>
-    <row r="395" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="395" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A395" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23694,7 +23694,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="396" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="396" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A396" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23715,7 +23715,7 @@
       </c>
       <c r="G396" s="4"/>
     </row>
-    <row r="397" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="397" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A397" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23738,7 +23738,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="398" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="398" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A398" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23761,7 +23761,7 @@
         <v>1104</v>
       </c>
     </row>
-    <row r="399" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="399" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A399" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23784,7 +23784,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="400" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="400" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A400" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23805,7 +23805,7 @@
       </c>
       <c r="G400" s="4"/>
     </row>
-    <row r="401" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="401" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A401" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23826,7 +23826,7 @@
       </c>
       <c r="G401" s="4"/>
     </row>
-    <row r="402" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="402" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A402" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23849,7 +23849,7 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="403" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="403" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A403" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23872,7 +23872,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="404" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="404" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A404" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23893,7 +23893,7 @@
       </c>
       <c r="G404" s="4"/>
     </row>
-    <row r="405" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="405" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A405" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23916,7 +23916,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="406" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="406" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A406" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23939,7 +23939,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="407" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="407" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A407" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23962,7 +23962,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="408" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="408" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A408" s="4" t="s">
         <v>1015</v>
       </c>
@@ -23983,7 +23983,7 @@
       </c>
       <c r="G408" s="4"/>
     </row>
-    <row r="409" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="409" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A409" s="4" t="s">
         <v>1015</v>
       </c>
@@ -24006,7 +24006,7 @@
         <v>1089</v>
       </c>
     </row>
-    <row r="410" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="410" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A410" s="4" t="s">
         <v>1015</v>
       </c>
@@ -24029,7 +24029,7 @@
         <v>1090</v>
       </c>
     </row>
-    <row r="411" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="411" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A411" s="4" t="s">
         <v>1015</v>
       </c>
@@ -24050,7 +24050,7 @@
       </c>
       <c r="G411" s="4"/>
     </row>
-    <row r="412" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="412" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A412" s="4" t="s">
         <v>1015</v>
       </c>
@@ -24073,7 +24073,7 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="413" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="413" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A413" s="4" t="s">
         <v>1015</v>
       </c>
@@ -24094,7 +24094,7 @@
       </c>
       <c r="G413" s="4"/>
     </row>
-    <row r="414" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="414" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A414" s="4" t="s">
         <v>1015</v>
       </c>
@@ -24117,7 +24117,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="415" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="415" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A415" s="4" t="s">
         <v>1015</v>
       </c>
@@ -24140,7 +24140,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="416" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="416" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A416" s="4" t="s">
         <v>1015</v>
       </c>
@@ -24163,7 +24163,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="417" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="417" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A417" s="4" t="s">
         <v>1015</v>
       </c>
@@ -24186,7 +24186,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="418" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="418" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A418" s="4" t="s">
         <v>1015</v>
       </c>
@@ -29455,7 +29455,7 @@
       </c>
       <c r="G660" s="4"/>
     </row>
-    <row r="661" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="661" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A661" s="4" t="s">
         <v>1003</v>
       </c>
@@ -29476,7 +29476,7 @@
       </c>
       <c r="G661" s="4"/>
     </row>
-    <row r="662" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="662" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A662" s="4" t="s">
         <v>1003</v>
       </c>
@@ -29499,7 +29499,7 @@
         <v>1065</v>
       </c>
     </row>
-    <row r="663" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="663" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A663" s="4" t="s">
         <v>1003</v>
       </c>
@@ -29520,7 +29520,7 @@
       </c>
       <c r="G663" s="4"/>
     </row>
-    <row r="664" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="664" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A664" s="4" t="s">
         <v>1003</v>
       </c>
@@ -29541,7 +29541,7 @@
       </c>
       <c r="G664" s="4"/>
     </row>
-    <row r="665" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="665" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A665" s="4" t="s">
         <v>1003</v>
       </c>
@@ -29562,7 +29562,7 @@
       </c>
       <c r="G665" s="4"/>
     </row>
-    <row r="666" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="666" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A666" s="4" t="s">
         <v>1003</v>
       </c>
@@ -31625,7 +31625,7 @@
       </c>
       <c r="G762" s="4"/>
     </row>
-    <row r="763" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="763" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A763" s="4" t="s">
         <v>1139</v>
       </c>
@@ -31646,7 +31646,7 @@
       </c>
       <c r="G763" s="4"/>
     </row>
-    <row r="764" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="764" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A764" s="4" t="s">
         <v>1139</v>
       </c>
@@ -31667,7 +31667,7 @@
       </c>
       <c r="G764" s="4"/>
     </row>
-    <row r="765" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="765" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A765" s="4" t="s">
         <v>1139</v>
       </c>
@@ -31688,7 +31688,7 @@
       </c>
       <c r="G765" s="4"/>
     </row>
-    <row r="766" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="766" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A766" s="4" t="s">
         <v>1139</v>
       </c>
@@ -33248,7 +33248,7 @@
   <autoFilter ref="A1:G837" xr:uid="{00000000-0009-0000-0000-00000A000000}">
     <filterColumn colId="2">
       <filters>
-        <filter val="Lithium"/>
+        <filter val="Tellurium"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -33349,7 +33349,7 @@
       <c r="B1" s="23" t="s">
         <v>1167</v>
       </c>
-      <c r="C1" s="204" t="s">
+      <c r="C1" s="190" t="s">
         <v>63</v>
       </c>
       <c r="D1" s="183"/>
@@ -33358,7 +33358,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="192" t="s">
+      <c r="A2" s="195" t="s">
         <v>76</v>
       </c>
       <c r="B2" s="177"/>
@@ -33685,8 +33685,8 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="193"/>
-      <c r="B27" s="194"/>
+      <c r="A27" s="196"/>
+      <c r="B27" s="197"/>
       <c r="C27" s="37" t="s">
         <v>1201</v>
       </c>
@@ -33698,10 +33698,10 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="195" t="s">
+      <c r="A28" s="198" t="s">
         <v>78</v>
       </c>
-      <c r="B28" s="196" t="s">
+      <c r="B28" s="199" t="s">
         <v>78</v>
       </c>
       <c r="C28" s="74" t="s">
@@ -33714,7 +33714,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="179"/>
-      <c r="B29" s="191"/>
+      <c r="B29" s="194"/>
       <c r="C29" s="21" t="s">
         <v>1204</v>
       </c>
@@ -33724,7 +33724,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="179"/>
-      <c r="B30" s="199" t="s">
+      <c r="B30" s="202" t="s">
         <v>1206</v>
       </c>
       <c r="C30" s="21" t="s">
@@ -33739,7 +33739,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="179"/>
-      <c r="B31" s="191"/>
+      <c r="B31" s="194"/>
       <c r="C31" s="21" t="s">
         <v>1204</v>
       </c>
@@ -33752,7 +33752,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="179"/>
-      <c r="B32" s="199" t="s">
+      <c r="B32" s="202" t="s">
         <v>1209</v>
       </c>
       <c r="C32" s="52" t="s">
@@ -33767,7 +33767,7 @@
     </row>
     <row r="33" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="179"/>
-      <c r="B33" s="198"/>
+      <c r="B33" s="201"/>
       <c r="C33" s="4" t="s">
         <v>1079</v>
       </c>
@@ -33778,7 +33778,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="179"/>
-      <c r="B34" s="198"/>
+      <c r="B34" s="201"/>
       <c r="C34" s="52" t="s">
         <v>1018</v>
       </c>
@@ -33789,7 +33789,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="179"/>
-      <c r="B35" s="191"/>
+      <c r="B35" s="194"/>
       <c r="C35" s="4" t="s">
         <v>1073</v>
       </c>
@@ -33802,7 +33802,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="179"/>
-      <c r="B36" s="199" t="s">
+      <c r="B36" s="202" t="s">
         <v>1216</v>
       </c>
       <c r="C36" s="21" t="s">
@@ -33817,7 +33817,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="179"/>
-      <c r="B37" s="198"/>
+      <c r="B37" s="201"/>
       <c r="C37" s="21" t="s">
         <v>1035</v>
       </c>
@@ -33830,7 +33830,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="179"/>
-      <c r="B38" s="198"/>
+      <c r="B38" s="201"/>
       <c r="C38" s="21" t="s">
         <v>1109</v>
       </c>
@@ -33843,7 +33843,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" s="179"/>
-      <c r="B39" s="191"/>
+      <c r="B39" s="194"/>
       <c r="C39" s="4" t="s">
         <v>1073</v>
       </c>
@@ -33854,7 +33854,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" s="179"/>
-      <c r="B40" s="201" t="s">
+      <c r="B40" s="203" t="s">
         <v>1222</v>
       </c>
       <c r="C40" s="21" t="s">
@@ -33869,7 +33869,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="179"/>
-      <c r="B41" s="198"/>
+      <c r="B41" s="201"/>
       <c r="C41" s="21" t="s">
         <v>1224</v>
       </c>
@@ -33882,7 +33882,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="179"/>
-      <c r="B42" s="198"/>
+      <c r="B42" s="201"/>
       <c r="C42" s="21" t="s">
         <v>1226</v>
       </c>
@@ -33895,7 +33895,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="179"/>
-      <c r="B43" s="198"/>
+      <c r="B43" s="201"/>
       <c r="C43" s="21" t="s">
         <v>182</v>
       </c>
@@ -33907,8 +33907,8 @@
       </c>
     </row>
     <row r="44" spans="1:5" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="194"/>
-      <c r="B44" s="202"/>
+      <c r="A44" s="197"/>
+      <c r="B44" s="204"/>
       <c r="C44" s="163" t="s">
         <v>1229</v>
       </c>
@@ -33920,10 +33920,10 @@
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="205" t="s">
+      <c r="A45" s="191" t="s">
         <v>84</v>
       </c>
-      <c r="B45" s="200"/>
+      <c r="B45" s="192"/>
       <c r="C45" s="152" t="s">
         <v>1145</v>
       </c>
@@ -33943,10 +33943,10 @@
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="197" t="s">
+      <c r="A47" s="200" t="s">
         <v>1233</v>
       </c>
-      <c r="B47" s="200"/>
+      <c r="B47" s="192"/>
       <c r="C47" s="49" t="s">
         <v>1234</v>
       </c>
@@ -33966,7 +33966,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" s="197" t="s">
+      <c r="A49" s="200" t="s">
         <v>89</v>
       </c>
       <c r="B49" s="169" t="s">
@@ -33983,7 +33983,7 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" s="198"/>
+      <c r="A50" s="201"/>
       <c r="B50" s="50" t="s">
         <v>1239</v>
       </c>
@@ -33998,8 +33998,8 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" s="198"/>
-      <c r="B51" s="203" t="s">
+      <c r="A51" s="201"/>
+      <c r="B51" s="205" t="s">
         <v>1242</v>
       </c>
       <c r="C51" s="21" t="s">
@@ -34008,20 +34008,20 @@
       <c r="D51" s="75" t="s">
         <v>1244</v>
       </c>
-      <c r="E51" s="190" t="s">
+      <c r="E51" s="193" t="s">
         <v>1245</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="191"/>
-      <c r="B52" s="191"/>
+      <c r="A52" s="194"/>
+      <c r="B52" s="194"/>
       <c r="C52" s="163" t="s">
         <v>1246</v>
       </c>
       <c r="D52" s="173" t="s">
         <v>1247</v>
       </c>
-      <c r="E52" s="191"/>
+      <c r="E52" s="194"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" s="170"/>
@@ -38867,8 +38867,8 @@
       <c r="A5" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="120">
-        <v>0</v>
+      <c r="B5" s="122">
+        <v>11850</v>
       </c>
       <c r="C5" s="4">
         <v>560</v>
@@ -38880,7 +38880,7 @@
         <v>11850</v>
       </c>
       <c r="F5" s="4">
-        <v>0</v>
+        <v>11850</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.2">
@@ -39264,10 +39264,12 @@
         <v>74</v>
       </c>
       <c r="D25" s="122">
-        <v>1</v>
+        <f>D21/4</f>
+        <v>219</v>
       </c>
       <c r="E25" s="122">
-        <v>1</v>
+        <f>E21/4</f>
+        <v>242.25</v>
       </c>
       <c r="F25" s="118">
         <v>1</v>
@@ -39870,11 +39872,11 @@
       <c r="A5" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="24">
-        <v>0</v>
+      <c r="B5" s="4">
+        <v>11850</v>
       </c>
       <c r="C5" s="4">
-        <v>0</v>
+        <v>11850</v>
       </c>
       <c r="D5" s="24">
         <v>0</v>
@@ -40761,7 +40763,8 @@
         <v>0</v>
       </c>
       <c r="G25" s="4">
-        <v>1</v>
+        <f>G21/4</f>
+        <v>173.75</v>
       </c>
       <c r="H25" s="4">
         <v>0</v>
@@ -41318,13 +41321,13 @@
         <v>51</v>
       </c>
       <c r="B38" s="24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C38" s="4">
         <v>20</v>
       </c>
       <c r="D38" s="24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E38" s="4">
         <v>0</v>
@@ -41832,15 +41835,15 @@
       <c r="A5" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="151">
-        <v>0</v>
+      <c r="B5" s="4">
+        <v>118500</v>
       </c>
       <c r="C5" s="151">
         <v>0</v>
       </c>
       <c r="D5" s="4"/>
-      <c r="E5" s="151">
-        <v>0</v>
+      <c r="E5" s="4">
+        <v>118500</v>
       </c>
       <c r="F5" s="151">
         <v>0</v>
@@ -42764,8 +42767,8 @@
         <v>0</v>
       </c>
       <c r="H25" s="4">
-        <f>1/70</f>
-        <v>1.4285714285714285E-2</v>
+        <f>H21/4</f>
+        <v>2.4821428571428572</v>
       </c>
       <c r="I25" s="4">
         <v>0</v>

</xml_diff>